<commit_message>
Completat code review + SonarQube review
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chich\OneDrive\Desktop\An III\An III Sem II\VVSS\Lab1\VVSS-czr-dar\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D5334FE-A706-4882-9988-61EB6A92124A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E5E6CB8-5F1E-4C48-8F04-EF237D114226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="4044" windowWidth="23256" windowHeight="12456" tabRatio="650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="4044" windowWidth="23256" windowHeight="12456" tabRatio="650" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="83">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -132,9 +132,6 @@
     <t>Tool-based Code Analysis</t>
   </si>
   <si>
-    <t>Effort to perform tool-based code analysis (hours):</t>
-  </si>
-  <si>
     <t>Porcar Cezar</t>
   </si>
   <si>
@@ -145,13 +142,634 @@
   </si>
   <si>
     <t>10.03.2025</t>
+  </si>
+  <si>
+    <t>C12</t>
+  </si>
+  <si>
+    <t>Product.java</t>
+  </si>
+  <si>
+    <t>C01</t>
+  </si>
+  <si>
+    <t>Order.java</t>
+  </si>
+  <si>
+    <t>C06</t>
+  </si>
+  <si>
+    <t>FileOrderRepository.java</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Gestiunea pretului total nu este actualizata la un add sau remove de item din comanda. Lista de iteme nu ar trebui sa poata fi modificata de oricine. Metoda setTotalPrice publica aduce probleme de securitate. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fix:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Returnam o copie a listei de items. Stergem metota setTotalPrice. Apelam computeTotalPrice de fiecare data cand un item este adaugat sau sters</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Atributul descriere lipseste din implementare </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fix:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Am adaugat atributul String descriere, constructor modificat, getters/setter, toString </t>
+    </r>
+  </si>
+  <si>
+    <t>C04</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Logica de extragere din fisier este fragila. Nu este tratat cazul in care citim din fisier o comanda fara items. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Fix: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>adaug un check pentru part[1] pentru a verifica existenta item-elor</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Atributele cantitate si stocMinim sunt declarate de tip double, constructorul cere parametri de tip int. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fix:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> actualizam constructorul sa ceara double</t>
+    </r>
+  </si>
+  <si>
+    <t>C07</t>
+  </si>
+  <si>
+    <t>CsvExporter.java</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Se srie in fisier text care nu este compatibil cu formatul csv, creeand un fisier "corupt" </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fix:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> scrierea in fisier strict a datelor in format csv</t>
+    </r>
+  </si>
+  <si>
+    <t>C09</t>
+  </si>
+  <si>
+    <t>CsvExporter.java/ReceiptGenerator.java</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Logica complexa si reduntanta la extragerea unui produs din comanda. Posibil IndexOutOfBoundsException. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fix:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> clasa OrderItem contine metoda getProduct, se va utiliza aceasta</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Conceptul de stocMinim nu este prezent in cerinte. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Fix: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>eliminarea urmelor de stocMinim</t>
+    </r>
+  </si>
+  <si>
+    <t>Stoc.java/FileStocRepository.java/StocValidator.java</t>
+  </si>
+  <si>
+    <t>C05</t>
+  </si>
+  <si>
+    <t>OrderService.java</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Metodele addItem si removeItem modifica direct lista de iteme, ocolind metodele din Order dedicate acestui lucru. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fix:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> apelarea metodelor corecte</t>
+    </r>
+  </si>
+  <si>
+    <t>Stoc.java/StocService.java</t>
+  </si>
+  <si>
+    <t>Services</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">nu este apelat nicio metoda de validate in nicio clasa Service. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Fix: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>adaugare apel de metode de validare</t>
+    </r>
+  </si>
+  <si>
+    <t>DrinkShopController.java</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Metoda onFinalizeOrder omite verificarea stocurilor inainte de a efectua comanta, cerinta prezenta in documentul de cerinte </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fix:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> adaugarea verificarii</t>
+    </r>
+  </si>
+  <si>
+    <t>AbstractRepository.java, 20</t>
+  </si>
+  <si>
+    <t>Unnecessary cat to "List"</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">return </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(List&lt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF16BAAC"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>E</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>&gt;)StreamSupport.</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>stream</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFC77DBB"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>entities</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">.values().spliterator(), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFCF8E6D"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>false</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>).toList();</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">return </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>StreamSupport.</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>stream</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFC77DBB"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>entities</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">.values().spliterator(), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFCF8E6D"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>false</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>).toList();</t>
+    </r>
+  </si>
+  <si>
+    <t>Generic name convention</t>
+  </si>
+  <si>
+    <t>Schimbare prea mica pentru a afecta aplicatia</t>
+  </si>
+  <si>
+    <t>AbstractRepository.java, 8</t>
+  </si>
+  <si>
+    <t>OrderValidator.java, 25</t>
+  </si>
+  <si>
+    <t>Use StringBuilder instead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                errors += e.getMessage();</t>
+  </si>
+  <si>
+    <t>bld.append( e.getMessage());</t>
+  </si>
+  <si>
+    <t>FileAbstractRepository.java, 12</t>
+  </si>
+  <si>
+    <t>Change visibility to "protected"</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">public </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF56A8F5"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>FileAbstractRepository</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(String fileName) {</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">protected </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF56A8F5"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>FileAbstractRepository</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(String fileName) {</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">if </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">(sb.length() &gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF2AACB8"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>) {</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">if </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(sb.isEmpty()) {</t>
+    </r>
+  </si>
+  <si>
+    <t>FileOrderRepository.java, 60</t>
+  </si>
+  <si>
+    <t>User .isEmpty() to check if StringBuilder is empty or not</t>
+  </si>
+  <si>
+    <t>Effort to perform tool-based code analysis (hours): 0.5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -242,6 +860,49 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FFBCBEC4"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FFCF8E6D"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF16BAAC"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FFBCBEC4"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FFC77DBB"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF56A8F5"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF2AACB8"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="5">
@@ -343,7 +1004,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -416,6 +1077,15 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -725,7 +1395,7 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.85546875" style="6"/>
     <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
@@ -737,7 +1407,7 @@
     <col min="11" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.75">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
@@ -748,7 +1418,7 @@
       <c r="I1" s="24"/>
       <c r="J1" s="24"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10">
       <c r="B2" s="26" t="s">
         <v>19</v>
       </c>
@@ -763,14 +1433,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
       <c r="I3" s="17"/>
       <c r="J3" s="17"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10">
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
@@ -784,7 +1454,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10">
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
@@ -798,7 +1468,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
@@ -806,14 +1476,14 @@
       <c r="D6" s="23"/>
       <c r="E6" s="23"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="23"/>
       <c r="E7" s="23"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -827,7 +1497,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -835,7 +1505,7 @@
       <c r="D10" s="1"/>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -844,7 +1514,7 @@
       <c r="D11" s="1"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
@@ -853,7 +1523,7 @@
       <c r="D12" s="1"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -862,7 +1532,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -871,7 +1541,7 @@
       <c r="D14" s="1"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -880,7 +1550,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -889,7 +1559,7 @@
       <c r="D16" s="1"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:5">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -898,7 +1568,7 @@
       <c r="D17" s="1"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -907,7 +1577,7 @@
       <c r="D18" s="3"/>
       <c r="E18" s="15"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -916,7 +1586,7 @@
       <c r="D19" s="3"/>
       <c r="E19" s="15"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:5">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -925,7 +1595,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -934,7 +1604,7 @@
       <c r="D21" s="3"/>
       <c r="E21" s="15"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -943,7 +1613,7 @@
       <c r="D22" s="3"/>
       <c r="E22" s="15"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -952,7 +1622,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="15"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -961,7 +1631,7 @@
       <c r="D24" s="3"/>
       <c r="E24" s="15"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -970,7 +1640,7 @@
       <c r="D25" s="3"/>
       <c r="E25" s="15"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:5">
       <c r="C27" s="11" t="s">
         <v>8</v>
       </c>
@@ -997,7 +1667,7 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.85546875" style="6"/>
     <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
@@ -1008,7 +1678,7 @@
     <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.75">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
@@ -1019,7 +1689,7 @@
       <c r="I1" s="24"/>
       <c r="J1" s="24"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10">
       <c r="B2" s="26" t="s">
         <v>18</v>
       </c>
@@ -1034,14 +1704,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
       <c r="I3" s="17"/>
       <c r="J3" s="17"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10">
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
@@ -1055,7 +1725,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10">
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
@@ -1069,7 +1739,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
@@ -1077,14 +1747,14 @@
       <c r="D6" s="23"/>
       <c r="E6" s="23"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="23"/>
       <c r="E7" s="23"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1098,7 +1768,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1106,7 +1776,7 @@
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1115,7 +1785,7 @@
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B26" si="0">B11+1</f>
         <v>3</v>
@@ -1124,7 +1794,7 @@
       <c r="D12" s="1"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1133,7 +1803,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1142,7 +1812,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1151,7 +1821,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1160,7 +1830,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:5">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1169,7 +1839,7 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1178,7 +1848,7 @@
       <c r="D18" s="1"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1187,7 +1857,7 @@
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:5">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1196,7 +1866,7 @@
       <c r="D20" s="1"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1205,7 +1875,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1214,7 +1884,7 @@
       <c r="D22" s="1"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1223,7 +1893,7 @@
       <c r="D23" s="1"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1232,7 +1902,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1241,7 +1911,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:5">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1250,7 +1920,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:5">
       <c r="C28" s="11" t="s">
         <v>8</v>
       </c>
@@ -1277,19 +1947,19 @@
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.85546875" style="6"/>
     <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
     <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
-    <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="30.5703125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="41" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="8" width="8.85546875" style="6"/>
     <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
     <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.75">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
@@ -1300,7 +1970,7 @@
       <c r="I1" s="24"/>
       <c r="J1" s="24"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10">
       <c r="B2" s="26" t="s">
         <v>17</v>
       </c>
@@ -1315,18 +1985,18 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
       <c r="I3" s="22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J3" s="17">
         <v>235</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10">
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
@@ -1338,13 +2008,13 @@
         <v>21</v>
       </c>
       <c r="I4" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J4" s="3">
         <v>235</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10">
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
@@ -1358,26 +2028,26 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E6" s="23"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E7" s="23"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1391,96 +2061,156 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="60">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="135">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="75">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C12" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="60">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="45">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="75">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="45">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="60">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C17" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="45">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="60">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1489,7 +2219,7 @@
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1498,7 +2228,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1507,7 +2237,7 @@
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1516,7 +2246,7 @@
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1525,7 +2255,7 @@
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1534,7 +2264,7 @@
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:5">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1543,7 +2273,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:5">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1552,7 +2282,7 @@
       <c r="D27" s="2"/>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:5">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1561,7 +2291,7 @@
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:5">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -1570,7 +2300,7 @@
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:5">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1579,12 +2309,14 @@
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:5">
       <c r="C32" s="11" t="s">
         <v>8</v>
       </c>
       <c r="D32" s="12"/>
-      <c r="E32" s="1"/>
+      <c r="E32" s="1">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1606,20 +2338,20 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.85546875" style="6"/>
     <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="26.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23.85546875" style="6" customWidth="1"/>
+    <col min="5" max="5" width="41.5703125" style="6" customWidth="1"/>
     <col min="6" max="6" width="16.5703125" style="6" customWidth="1"/>
     <col min="7" max="8" width="8.85546875" style="6"/>
     <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
     <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.75">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
@@ -1630,7 +2362,7 @@
       <c r="I1" s="24"/>
       <c r="J1" s="24"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10">
       <c r="B2" s="26" t="s">
         <v>31</v>
       </c>
@@ -1645,14 +2377,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
       <c r="I3" s="17"/>
       <c r="J3" s="17"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10">
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
@@ -1664,7 +2396,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10">
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
@@ -1676,7 +2408,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>1</v>
@@ -1685,7 +2417,7 @@
       <c r="E6" s="23"/>
       <c r="F6" s="20"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1702,56 +2434,94 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="108">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C10" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="38" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="38" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="45">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>67</v>
+      </c>
       <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F11" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C12" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="39" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="30">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C13" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" s="37" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="60">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C14" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>78</v>
+      </c>
+      <c r="F14" s="37" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1761,7 +2531,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1771,7 +2541,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1781,7 +2551,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1791,7 +2561,7 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1801,7 +2571,7 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1811,7 +2581,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1821,7 +2591,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1831,7 +2601,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1841,7 +2611,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1851,7 +2621,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1861,7 +2631,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1871,7 +2641,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1881,7 +2651,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1891,7 +2661,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -1901,7 +2671,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1911,15 +2681,15 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6">
       <c r="C32" s="35" t="s">
-        <v>32</v>
+        <v>82</v>
       </c>
       <c r="D32" s="36"/>
       <c r="E32" s="36"/>
       <c r="F32" s="18"/>
     </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="6:6">
       <c r="F35" s="21"/>
     </row>
   </sheetData>

</xml_diff>